<commit_message>
HUD updates, sound tweaks
Made default system mouse pointer return when over certain HUD areas where selection is needed.
Shortened torpedo life span by 1/3 to reduce accidental hits on off-screen enemies.
Edited torpedo shot sound to be shorter.
</commit_message>
<xml_diff>
--- a/sprite_sheet.xlsx
+++ b/sprite_sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nthnl\Desktop\Code\Flashtrek-2.0-Godot-4.4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05146CBA-BE6C-496D-BA57-70669290DF8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CBBE4B2-297B-4B3C-A695-40A7122CBBD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9480D77A-E5C1-4096-97D1-11AE8DADC1A6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9480D77A-E5C1-4096-97D1-11AE8DADC1A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprites" sheetId="1" r:id="rId1"/>
@@ -419,16 +419,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>75520</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>200704</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>7485</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>37418</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>545645</xdr:colOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>477610</xdr:colOff>
       <xdr:row>71</xdr:row>
-      <xdr:rowOff>36737</xdr:rowOff>
+      <xdr:rowOff>172808</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -457,7 +457,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14730413" y="200704"/>
+          <a:off x="15274699" y="336775"/>
           <a:ext cx="11491911" cy="21090390"/>
         </a:xfrm>
         <a:prstGeom prst="rect">

</xml_diff>

<commit_message>
Settings Menu state saves
Fixed not being able to complete cargo delivery missions at correct planet.
Set settings menu state to load and save user settings.
</commit_message>
<xml_diff>
--- a/sprite_sheet.xlsx
+++ b/sprite_sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nthnl\Desktop\Code\Flashtrek-2.0-Godot-4.4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CBBE4B2-297B-4B3C-A695-40A7122CBBD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38E779C4-C3F1-4AB2-B20D-0159C6F61777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9480D77A-E5C1-4096-97D1-11AE8DADC1A6}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9480D77A-E5C1-4096-97D1-11AE8DADC1A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprites" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
New Ship Menu (WIP), player shooting change
Player can now aim toward mouse instead of only directly forward. Greatly increases aiming ease.
Added new WIP ship status menu. Currently not wired or in-game.
</commit_message>
<xml_diff>
--- a/sprite_sheet.xlsx
+++ b/sprite_sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nthnl\Desktop\Code\Flashtrek-2.0-Godot-4.4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38E779C4-C3F1-4AB2-B20D-0159C6F61777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{307699B1-BD73-4125-A6C9-E36659E5DDA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9480D77A-E5C1-4096-97D1-11AE8DADC1A6}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="97">
   <si>
     <t>Merchantman</t>
   </si>
@@ -327,9 +327,6 @@
   </si>
   <si>
     <t>X</t>
-  </si>
-  <si>
-    <t>Y</t>
   </si>
 </sst>
 </file>
@@ -787,7 +784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89A46386-5A4D-4B73-8EAB-C9B2C9DD0814}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultRowHeight="24" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -1180,11 +1177,6 @@
         <v>81</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.4">
-      <c r="A16" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>